<commit_message>
Finalize phase 3 visual overhaul: full red theme, animated video modal, smooth card expansion, header polish, finance rebuild, and module restructuring
</commit_message>
<xml_diff>
--- a/islami-assistant-web/public/data/اسماء الموظفين وكلمات السر .xlsx
+++ b/islami-assistant-web/public/data/اسماء الموظفين وكلمات السر .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLACK-DIAMOND\Desktop\islami Assistant\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLACK-DIAMOND\Desktop\islami Assistant\islami-assistant-web\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7EF7FBE-59FA-45B7-A567-FB3D32A1E533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4BFEC1-BD23-4475-96C0-0EC11E1ECDF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,28 +20,14 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>الاسم</t>
-  </si>
-  <si>
-    <t>مركز الاتصال</t>
   </si>
   <si>
     <t>ينال عساف</t>
@@ -158,13 +144,13 @@
     <t>رغد شراقة</t>
   </si>
   <si>
-    <t>User</t>
+    <t xml:space="preserve">انس حسن </t>
   </si>
   <si>
-    <t>password</t>
+    <t xml:space="preserve">اسم المستخدم </t>
   </si>
   <si>
-    <t xml:space="preserve">انس حسن </t>
+    <t xml:space="preserve">كلمة المرور </t>
   </si>
 </sst>
 </file>
@@ -180,13 +166,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="15"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="18"/>
       <color theme="1"/>
@@ -194,8 +173,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,29 +190,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -260,58 +231,28 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="2"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="عادي" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -589,515 +530,474 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1001"/>
+  <dimension ref="A1:C989"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="36.5703125" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:3" s="5" customFormat="1" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="8"/>
-    </row>
-    <row r="3" spans="1:3" ht="19.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="6" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="2">
+        <v>88001</v>
+      </c>
+      <c r="C2" s="2">
+        <v>88001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2">
+        <v>5016</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5016</v>
+      </c>
     </row>
     <row r="4" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
-        <v>88001</v>
-      </c>
-      <c r="B4" s="5" t="str">
-        <f>"pass@"&amp;A4</f>
-        <v>pass@88001</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B4" s="2">
+        <v>88002</v>
+      </c>
+      <c r="C4" s="2">
+        <v>88002</v>
+      </c>
     </row>
     <row r="5" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
-        <v>5016</v>
-      </c>
-      <c r="B5" s="5" t="str">
-        <f>"pass@"&amp;A5</f>
-        <v>pass@5016</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>42</v>
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>88003</v>
+      </c>
+      <c r="C5" s="2">
+        <v>88003</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A6" s="5">
-        <v>88002</v>
-      </c>
-      <c r="B6" s="5" t="str">
-        <f t="shared" ref="B6:B43" si="0">"pass@"&amp;A6</f>
-        <v>pass@88002</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>3</v>
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <v>88004</v>
+      </c>
+      <c r="C6" s="2">
+        <v>88004</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A7" s="5">
-        <v>88003</v>
-      </c>
-      <c r="B7" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88003</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>4</v>
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2">
+        <v>88005</v>
+      </c>
+      <c r="C7" s="2">
+        <v>88005</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
-        <v>88004</v>
-      </c>
-      <c r="B8" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88004</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>5</v>
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <v>88006</v>
+      </c>
+      <c r="C8" s="2">
+        <v>88006</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
-        <v>88005</v>
-      </c>
-      <c r="B9" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88005</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>6</v>
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2">
+        <v>88007</v>
+      </c>
+      <c r="C9" s="2">
+        <v>88007</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
-        <v>88006</v>
-      </c>
-      <c r="B10" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88006</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>7</v>
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2">
+        <v>88008</v>
+      </c>
+      <c r="C10" s="2">
+        <v>88008</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
-        <v>88007</v>
-      </c>
-      <c r="B11" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88007</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>8</v>
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2">
+        <v>88009</v>
+      </c>
+      <c r="C11" s="2">
+        <v>88009</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A12" s="5">
-        <v>88008</v>
-      </c>
-      <c r="B12" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88008</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>9</v>
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2">
+        <v>88010</v>
+      </c>
+      <c r="C12" s="2">
+        <v>88010</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A13" s="5">
-        <v>88009</v>
-      </c>
-      <c r="B13" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88009</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>10</v>
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <v>88011</v>
+      </c>
+      <c r="C13" s="2">
+        <v>88011</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A14" s="5">
-        <v>88010</v>
-      </c>
-      <c r="B14" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88010</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>11</v>
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2">
+        <v>88012</v>
+      </c>
+      <c r="C14" s="2">
+        <v>88012</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A15" s="5">
-        <v>88011</v>
-      </c>
-      <c r="B15" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88011</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>12</v>
+      <c r="A15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2">
+        <v>88013</v>
+      </c>
+      <c r="C15" s="2">
+        <v>88013</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A16" s="5">
-        <v>88012</v>
-      </c>
-      <c r="B16" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88012</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>13</v>
+      <c r="A16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2">
+        <v>88014</v>
+      </c>
+      <c r="C16" s="2">
+        <v>88014</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A17" s="5">
-        <v>88013</v>
-      </c>
-      <c r="B17" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88013</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>14</v>
+      <c r="A17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2">
+        <v>88015</v>
+      </c>
+      <c r="C17" s="2">
+        <v>88015</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A18" s="5">
-        <v>88014</v>
-      </c>
-      <c r="B18" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88014</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>15</v>
+      <c r="A18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2">
+        <v>88016</v>
+      </c>
+      <c r="C18" s="2">
+        <v>88016</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A19" s="5">
-        <v>88015</v>
-      </c>
-      <c r="B19" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88015</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>16</v>
+      <c r="A19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2">
+        <v>88017</v>
+      </c>
+      <c r="C19" s="2">
+        <v>88017</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
-        <v>88016</v>
-      </c>
-      <c r="B20" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88016</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>17</v>
+      <c r="A20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2">
+        <v>88018</v>
+      </c>
+      <c r="C20" s="2">
+        <v>88018</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A21" s="5">
-        <v>88017</v>
-      </c>
-      <c r="B21" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88017</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>18</v>
+      <c r="A21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2">
+        <v>88019</v>
+      </c>
+      <c r="C21" s="2">
+        <v>88019</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A22" s="5">
-        <v>88018</v>
-      </c>
-      <c r="B22" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88018</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>19</v>
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2">
+        <v>88020</v>
+      </c>
+      <c r="C22" s="2">
+        <v>88020</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A23" s="5">
-        <v>88019</v>
-      </c>
-      <c r="B23" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88019</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>20</v>
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2">
+        <v>88021</v>
+      </c>
+      <c r="C23" s="2">
+        <v>88021</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A24" s="5">
-        <v>88020</v>
-      </c>
-      <c r="B24" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88020</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>21</v>
+      <c r="A24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2">
+        <v>88022</v>
+      </c>
+      <c r="C24" s="2">
+        <v>88022</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A25" s="5">
-        <v>88021</v>
-      </c>
-      <c r="B25" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88021</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>22</v>
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2">
+        <v>88023</v>
+      </c>
+      <c r="C25" s="2">
+        <v>88023</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A26" s="5">
-        <v>88022</v>
-      </c>
-      <c r="B26" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88022</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>23</v>
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2">
+        <v>88024</v>
+      </c>
+      <c r="C26" s="2">
+        <v>88024</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A27" s="5">
-        <v>88023</v>
-      </c>
-      <c r="B27" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88023</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>24</v>
+      <c r="A27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2">
+        <v>88025</v>
+      </c>
+      <c r="C27" s="2">
+        <v>88025</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A28" s="5">
-        <v>88024</v>
-      </c>
-      <c r="B28" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88024</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>25</v>
+      <c r="A28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2">
+        <v>88026</v>
+      </c>
+      <c r="C28" s="2">
+        <v>88026</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>88025</v>
-      </c>
-      <c r="B29" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88025</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="A29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2">
+        <v>88027</v>
+      </c>
+      <c r="C29" s="2">
+        <v>88027</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2">
+        <v>88028</v>
+      </c>
+      <c r="C30" s="2">
+        <v>88028</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2">
+        <v>88029</v>
+      </c>
+      <c r="C31" s="2">
+        <v>88029</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2">
+        <v>88030</v>
+      </c>
+      <c r="C32" s="2">
+        <v>88030</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2">
+        <v>88031</v>
+      </c>
+      <c r="C33" s="2">
+        <v>88031</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="2">
+        <v>88032</v>
+      </c>
+      <c r="C34" s="2">
+        <v>88032</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="2">
+        <v>88033</v>
+      </c>
+      <c r="C35" s="2">
+        <v>88033</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" s="2">
+        <v>88034</v>
+      </c>
+      <c r="C36" s="2">
+        <v>88034</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="2">
+        <v>88035</v>
+      </c>
+      <c r="C37" s="2">
+        <v>88035</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="2">
+        <v>88036</v>
+      </c>
+      <c r="C38" s="2">
+        <v>88036</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" s="2">
+        <v>88037</v>
+      </c>
+      <c r="C39" s="2">
+        <v>88037</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A30" s="5">
-        <v>88026</v>
-      </c>
-      <c r="B30" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88026</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A31" s="5">
-        <v>88027</v>
-      </c>
-      <c r="B31" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88027</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A32" s="5">
-        <v>88028</v>
-      </c>
-      <c r="B32" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88028</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A33" s="5">
-        <v>88029</v>
-      </c>
-      <c r="B33" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88029</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A34" s="5">
-        <v>88030</v>
-      </c>
-      <c r="B34" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88030</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A35" s="5">
-        <v>88031</v>
-      </c>
-      <c r="B35" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88031</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A36" s="5">
-        <v>88032</v>
-      </c>
-      <c r="B36" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88032</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A37" s="5">
-        <v>88033</v>
-      </c>
-      <c r="B37" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88033</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A38" s="5">
-        <v>88034</v>
-      </c>
-      <c r="B38" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88034</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A39" s="5">
-        <v>88035</v>
-      </c>
-      <c r="B39" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88035</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A40" s="5">
-        <v>88036</v>
-      </c>
-      <c r="B40" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88036</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>37</v>
+      <c r="B40" s="2">
+        <v>88038</v>
+      </c>
+      <c r="C40" s="2">
+        <v>88038</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A41" s="5">
-        <v>88037</v>
-      </c>
-      <c r="B41" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88037</v>
-      </c>
-      <c r="C41" s="5" t="s">
+      <c r="A41" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A42" s="5">
-        <v>88038</v>
-      </c>
-      <c r="B42" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88038</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A43" s="5">
+      <c r="B41" s="2">
         <v>88039</v>
       </c>
-      <c r="B43" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>pass@88039</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>39</v>
-      </c>
+      <c r="C41" s="2">
+        <v>88039</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
@@ -1105,14 +1005,14 @@
       <c r="C44" s="1"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="2"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="2"/>
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="2"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="2"/>
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
@@ -5829,72 +5729,7 @@
       <c r="B989" s="1"/>
       <c r="C989" s="1"/>
     </row>
-    <row r="990" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A990" s="1"/>
-      <c r="B990" s="1"/>
-      <c r="C990" s="1"/>
-    </row>
-    <row r="991" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A991" s="1"/>
-      <c r="B991" s="1"/>
-      <c r="C991" s="1"/>
-    </row>
-    <row r="992" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A992" s="1"/>
-      <c r="B992" s="1"/>
-      <c r="C992" s="1"/>
-    </row>
-    <row r="993" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A993" s="1"/>
-      <c r="B993" s="1"/>
-      <c r="C993" s="1"/>
-    </row>
-    <row r="994" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A994" s="1"/>
-      <c r="B994" s="1"/>
-      <c r="C994" s="1"/>
-    </row>
-    <row r="995" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A995" s="1"/>
-      <c r="B995" s="1"/>
-      <c r="C995" s="1"/>
-    </row>
-    <row r="996" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A996" s="1"/>
-      <c r="B996" s="1"/>
-      <c r="C996" s="1"/>
-    </row>
-    <row r="997" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A997" s="1"/>
-      <c r="B997" s="1"/>
-      <c r="C997" s="1"/>
-    </row>
-    <row r="998" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A998" s="1"/>
-      <c r="B998" s="1"/>
-      <c r="C998" s="1"/>
-    </row>
-    <row r="999" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A999" s="1"/>
-      <c r="B999" s="1"/>
-      <c r="C999" s="1"/>
-    </row>
-    <row r="1000" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1000" s="1"/>
-      <c r="B1000" s="1"/>
-      <c r="C1000" s="1"/>
-    </row>
-    <row r="1001" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1001" s="1"/>
-      <c r="B1001" s="1"/>
-      <c r="C1001" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Wipe finance rates and sync new unique index schema
</commit_message>
<xml_diff>
--- a/islami-assistant-web/public/data/اسماء الموظفين وكلمات السر .xlsx
+++ b/islami-assistant-web/public/data/اسماء الموظفين وكلمات السر .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLACK-DIAMOND\Desktop\islami Assistant\islami-assistant-web\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69E5E78-7B4D-4C6B-9F71-6A7DCA9FCBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D38C0A-A1A6-4F78-BAC7-B3F5F29F6F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,123 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>الاسم</t>
   </si>
   <si>
     <t>ينال عساف</t>
-  </si>
-  <si>
-    <t>ابراهيم الدغيلي</t>
-  </si>
-  <si>
-    <t>محمود أبو دية</t>
-  </si>
-  <si>
-    <t>هشام براو</t>
-  </si>
-  <si>
-    <t>محمد الرفاعي</t>
-  </si>
-  <si>
-    <t>احمد ملكاوي</t>
-  </si>
-  <si>
-    <t>اياد سعادات</t>
-  </si>
-  <si>
-    <t>براء الدبس</t>
-  </si>
-  <si>
-    <t>عمر أبو حفيظة</t>
-  </si>
-  <si>
-    <t>راشد بني عطا</t>
-  </si>
-  <si>
-    <t>منذر الغول</t>
-  </si>
-  <si>
-    <t>طارق الغول</t>
-  </si>
-  <si>
-    <t>عمر جاد الله</t>
-  </si>
-  <si>
-    <t>عوني الكوز</t>
-  </si>
-  <si>
-    <t>علاء عيسى</t>
-  </si>
-  <si>
-    <t>علي عاشور</t>
-  </si>
-  <si>
-    <t>احمد أبو حنان</t>
-  </si>
-  <si>
-    <t>محمد التيالخة</t>
-  </si>
-  <si>
-    <t>صهيب الشوبكي</t>
-  </si>
-  <si>
-    <t>عبدالله فتايلي</t>
-  </si>
-  <si>
-    <t>عبادة السلمي</t>
-  </si>
-  <si>
-    <t>سند حماد</t>
-  </si>
-  <si>
-    <t>فايز إبراهيم</t>
-  </si>
-  <si>
-    <t>عبد الله العسس</t>
-  </si>
-  <si>
-    <t>محمد محمود</t>
-  </si>
-  <si>
-    <t>احمد عشا</t>
-  </si>
-  <si>
-    <t>مروة صدقة</t>
-  </si>
-  <si>
-    <t>سلام الغول</t>
-  </si>
-  <si>
-    <t>بيسان الملاد</t>
-  </si>
-  <si>
-    <t>مرام القنبر</t>
-  </si>
-  <si>
-    <t>عفاف عودة</t>
-  </si>
-  <si>
-    <t>سارة الأطرش</t>
-  </si>
-  <si>
-    <t>رغد الشروف</t>
-  </si>
-  <si>
-    <t>رزان العلاوي</t>
-  </si>
-  <si>
-    <t>حنان قرينه</t>
-  </si>
-  <si>
-    <t>الاء حماد</t>
-  </si>
-  <si>
-    <t>محمد العضايلة</t>
-  </si>
-  <si>
-    <t>رغد شراقة</t>
   </si>
   <si>
     <t xml:space="preserve">انس حسن </t>
@@ -552,13 +441,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
@@ -572,12 +461,12 @@
         <v>88001</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>5016</v>
@@ -586,540 +475,236 @@
         <v>5016</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2">
-        <v>88002</v>
-      </c>
-      <c r="C4" s="2">
-        <v>88002</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2">
-        <v>88003</v>
-      </c>
-      <c r="C5" s="2">
-        <v>88003</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2">
-        <v>88004</v>
-      </c>
-      <c r="C6" s="2">
-        <v>88004</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2">
-        <v>88005</v>
-      </c>
-      <c r="C7" s="2">
-        <v>88005</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2">
-        <v>88006</v>
-      </c>
-      <c r="C8" s="2">
-        <v>88006</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
-        <v>88007</v>
-      </c>
-      <c r="C9" s="2">
-        <v>88007</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>43</v>
-      </c>
+    </row>
+    <row r="4" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2">
-        <v>88008</v>
-      </c>
-      <c r="C10" s="2">
-        <v>88008</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2">
-        <v>88009</v>
-      </c>
-      <c r="C11" s="2">
-        <v>88009</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="2">
-        <v>88010</v>
-      </c>
-      <c r="C12" s="2">
-        <v>88010</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2">
-        <v>88011</v>
-      </c>
-      <c r="C13" s="2">
-        <v>88011</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2">
-        <v>88012</v>
-      </c>
-      <c r="C14" s="2">
-        <v>88012</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="2">
-        <v>88013</v>
-      </c>
-      <c r="C15" s="2">
-        <v>88013</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="2">
-        <v>88014</v>
-      </c>
-      <c r="C16" s="2">
-        <v>88014</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="2">
-        <v>88015</v>
-      </c>
-      <c r="C17" s="2">
-        <v>88015</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="2">
-        <v>88016</v>
-      </c>
-      <c r="C18" s="2">
-        <v>88016</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="2">
-        <v>88017</v>
-      </c>
-      <c r="C19" s="2">
-        <v>88017</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="2">
-        <v>88018</v>
-      </c>
-      <c r="C20" s="2">
-        <v>88018</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="2">
-        <v>88019</v>
-      </c>
-      <c r="C21" s="2">
-        <v>88019</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2">
-        <v>88020</v>
-      </c>
-      <c r="C22" s="2">
-        <v>88020</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="2">
-        <v>88021</v>
-      </c>
-      <c r="C23" s="2">
-        <v>88021</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" s="2">
-        <v>88022</v>
-      </c>
-      <c r="C24" s="2">
-        <v>88022</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" s="2">
-        <v>88023</v>
-      </c>
-      <c r="C25" s="2">
-        <v>88023</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26" s="2">
-        <v>88024</v>
-      </c>
-      <c r="C26" s="2">
-        <v>88024</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="2">
-        <v>88025</v>
-      </c>
-      <c r="C27" s="2">
-        <v>88025</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="2">
-        <v>88026</v>
-      </c>
-      <c r="C28" s="2">
-        <v>88026</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="2">
-        <v>88027</v>
-      </c>
-      <c r="C29" s="2">
-        <v>88027</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B30" s="2">
-        <v>88028</v>
-      </c>
-      <c r="C30" s="2">
-        <v>88028</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
     </row>
     <row r="31" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2">
-        <v>88029</v>
-      </c>
-      <c r="C31" s="2">
-        <v>88029</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
     </row>
     <row r="32" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="2">
-        <v>88030</v>
-      </c>
-      <c r="C32" s="2">
-        <v>88030</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
     </row>
     <row r="33" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="2">
-        <v>88031</v>
-      </c>
-      <c r="C33" s="2">
-        <v>88031</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="2">
-        <v>88032</v>
-      </c>
-      <c r="C34" s="2">
-        <v>88032</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B35" s="2">
-        <v>88033</v>
-      </c>
-      <c r="C35" s="2">
-        <v>88033</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B36" s="2">
-        <v>88034</v>
-      </c>
-      <c r="C36" s="2">
-        <v>88034</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37" s="2">
-        <v>88035</v>
-      </c>
-      <c r="C37" s="2">
-        <v>88035</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B38" s="2">
-        <v>88036</v>
-      </c>
-      <c r="C38" s="2">
-        <v>88036</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B39" s="2">
-        <v>88037</v>
-      </c>
-      <c r="C39" s="2">
-        <v>88037</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B40" s="2">
-        <v>88038</v>
-      </c>
-      <c r="C40" s="2">
-        <v>88038</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
     </row>
     <row r="41" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B41" s="2">
-        <v>88039</v>
-      </c>
-      <c r="C41" s="2">
-        <v>88039</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>

</xml_diff>